<commit_message>
feat: complete real docking screening of 90 compounds and functional mechanism ranking
</commit_message>
<xml_diff>
--- a/03_DNA_Docking_Aim1/ranking_dna_binding_aim1.xlsx
+++ b/03_DNA_Docking_Aim1/ranking_dna_binding_aim1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M96"/>
+  <dimension ref="A1:M91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,7 +436,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Mechanism_Target</t>
+          <t>Functional_Mechanism</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -503,7 +503,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Aim 1: Minor Groove Binder</t>
+          <t>Aim 1: Minor Groove Specialist</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -527,13 +527,13 @@
         <v>3</v>
       </c>
       <c r="I2" t="n">
-        <v>-10.1</v>
+        <v>-8.699999999999999</v>
       </c>
       <c r="J2" t="n">
         <v>0.199</v>
       </c>
       <c r="K2" t="n">
-        <v>2.01</v>
+        <v>1.73</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -554,7 +554,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Aim 1: Minor Groove Binder</t>
+          <t>Aim 1: Minor Groove Specialist</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -578,13 +578,13 @@
         <v>4</v>
       </c>
       <c r="I3" t="n">
-        <v>-10.05</v>
+        <v>-8.699999999999999</v>
       </c>
       <c r="J3" t="n">
         <v>0.188</v>
       </c>
       <c r="K3" t="n">
-        <v>1.89</v>
+        <v>1.64</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
@@ -600,42 +600,42 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CHEMBL98244</t>
+          <t>CHEMBL163452</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Aim 1: Minor Groove Binder</t>
+          <t>Aim 1: Minor Groove Specialist</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Cc1nc2cc(-c3nc4cc(-c5nc6cc(-c7ccccc7)ccc6[nH]5)ccc4[nH]3)ccc2[nH]1</t>
+          <t>c1ccc(-c2ccc3[nH]c(-c4ccc5[nH]c(-c6ccc7nccnc7c6)nc5c4)nc3c2)cc1</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>440.51</v>
+        <v>438.49</v>
       </c>
       <c r="E4" t="n">
-        <v>6.62</v>
+        <v>6.38</v>
       </c>
       <c r="F4" t="n">
-        <v>86.04000000000001</v>
+        <v>83.14</v>
       </c>
       <c r="G4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I4" t="n">
-        <v>-9.800000000000001</v>
+        <v>-8.300000000000001</v>
       </c>
       <c r="J4" t="n">
-        <v>0.227</v>
+        <v>0.228</v>
       </c>
       <c r="K4" t="n">
-        <v>2.22</v>
+        <v>1.89</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -651,42 +651,42 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CHEMBL163452</t>
+          <t>CHEMBL98244</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Aim 1: Minor Groove Binder</t>
+          <t>Aim 1: Minor Groove Specialist</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>c1ccc(-c2ccc3[nH]c(-c4ccc5[nH]c(-c6ccc7nccnc7c6)nc5c4)nc3c2)cc1</t>
+          <t>Cc1nc2cc(-c3nc4cc(-c5nc6cc(-c7ccccc7)ccc6[nH]5)ccc4[nH]3)ccc2[nH]1</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>438.49</v>
+        <v>440.51</v>
       </c>
       <c r="E5" t="n">
-        <v>6.38</v>
+        <v>6.62</v>
       </c>
       <c r="F5" t="n">
-        <v>83.14</v>
+        <v>86.04000000000001</v>
       </c>
       <c r="G5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I5" t="n">
-        <v>-9.800000000000001</v>
+        <v>-8.300000000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>0.228</v>
+        <v>0.227</v>
       </c>
       <c r="K5" t="n">
-        <v>2.23</v>
+        <v>1.88</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
@@ -702,97 +702,97 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CHEMBL333953</t>
+          <t>CHEMBL1779470</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Aim 1: Minor Groove Binder</t>
+          <t>Aim 3: Dual-Action Lead</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>c1ccc2[nH]c(-c3ccc4[nH]c(-c5ccc6[nH]cnc6c5)nc4c3)nc2c1</t>
+          <t>O=c1cc(-c2ccc(O)c(-c3cc(-c4cc(=O)c5c(O)cc(O)cc5o4)ccc3O)c2)oc2cc(O)cc(O)c12</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>350.39</v>
+        <v>538.46</v>
       </c>
       <c r="E6" t="n">
-        <v>4.65</v>
+        <v>5.13</v>
       </c>
       <c r="F6" t="n">
-        <v>86.04000000000001</v>
+        <v>181.8</v>
       </c>
       <c r="G6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H6" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="I6" t="n">
-        <v>-9.5</v>
+        <v>-7.9</v>
       </c>
       <c r="J6" t="n">
-        <v>0.285</v>
+        <v>3.343</v>
       </c>
       <c r="K6" t="n">
-        <v>2.71</v>
+        <v>26.41</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>CHECK</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CHEMBL1672849</t>
+          <t>CHEMBL4847220</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Aim 1: Minor Groove Binder</t>
+          <t>Aim 3: Dual-Action Lead</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>c1ccc(-c2ccc3[nH]c(-c4ccc5nc(-c6ccccc6)[nH]c5c4)nc3c2)cc1</t>
+          <t>O=c1cc(-c2cccc(-c3c(O)cc(O)c4c(=O)cc(-c5ccc(O)c(O)c5)oc34)c2)oc2cc(O)cc(O)c12</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>386.46</v>
+        <v>538.46</v>
       </c>
       <c r="E7" t="n">
-        <v>6.44</v>
+        <v>5.13</v>
       </c>
       <c r="F7" t="n">
-        <v>57.36</v>
+        <v>181.8</v>
       </c>
       <c r="G7" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H7" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="I7" t="n">
-        <v>-9.449999999999999</v>
+        <v>-7.9</v>
       </c>
       <c r="J7" t="n">
-        <v>0.259</v>
+        <v>3.343</v>
       </c>
       <c r="K7" t="n">
-        <v>2.45</v>
+        <v>26.41</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -804,27 +804,27 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CHEMBL1683055</t>
+          <t>CHEMBL1927181</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Aim 1: Minor Groove Binder</t>
+          <t>Aim 1: Minor Groove Specialist</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Nc1nc2ccc(-c3ccc4nc5ccccc5nc4c3)cc2[nH]1</t>
+          <t>Cc1ccc(C(=O)Nc2nc3ccc(-c4ccc5nc6ccccc6nc5c4)cc3[nH]2)cc1</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>311.35</v>
+        <v>429.48</v>
       </c>
       <c r="E8" t="n">
-        <v>3.91</v>
+        <v>5.89</v>
       </c>
       <c r="F8" t="n">
-        <v>80.48</v>
+        <v>83.56</v>
       </c>
       <c r="G8" t="n">
         <v>2</v>
@@ -833,13 +833,13 @@
         <v>4</v>
       </c>
       <c r="I8" t="n">
-        <v>-9.199999999999999</v>
+        <v>-7.9</v>
       </c>
       <c r="J8" t="n">
-        <v>0.482</v>
+        <v>0.233</v>
       </c>
       <c r="K8" t="n">
-        <v>4.43</v>
+        <v>1.84</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
@@ -848,49 +848,49 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>CHECK</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CHEMBL3793039</t>
+          <t>CHEMBL333953</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Aim 1: Minor Groove Binder</t>
+          <t>Aim 1: Minor Groove Specialist</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>c1cc(-c2nc3ccccc3[nH]2)cc(-c2nc3ccccc3[nH]2)c1</t>
+          <t>c1ccc2[nH]c(-c3ccc4[nH]c(-c5ccc6[nH]cnc6c5)nc4c3)nc2c1</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>310.36</v>
+        <v>350.39</v>
       </c>
       <c r="E9" t="n">
-        <v>4.77</v>
+        <v>4.65</v>
       </c>
       <c r="F9" t="n">
-        <v>57.36</v>
+        <v>86.04000000000001</v>
       </c>
       <c r="G9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I9" t="n">
-        <v>-9.15</v>
+        <v>-7.9</v>
       </c>
       <c r="J9" t="n">
-        <v>0.322</v>
+        <v>0.285</v>
       </c>
       <c r="K9" t="n">
-        <v>2.95</v>
+        <v>2.25</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
@@ -906,42 +906,42 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CHEMBL367729</t>
+          <t>CHEMBL1672849</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Aim 1: Minor Groove Binder</t>
+          <t>Aim 1: Minor Groove Specialist</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>N#Cc1ccc2[nH]c(-c3ccc4[nH]c(-c5ccccc5)nc4c3)nc2c1</t>
+          <t>c1ccc(-c2ccc3[nH]c(-c4ccc5nc(-c6ccccc6)[nH]c5c4)nc3c2)cc1</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>335.37</v>
+        <v>386.46</v>
       </c>
       <c r="E10" t="n">
-        <v>4.64</v>
+        <v>6.44</v>
       </c>
       <c r="F10" t="n">
-        <v>81.15000000000001</v>
+        <v>57.36</v>
       </c>
       <c r="G10" t="n">
         <v>2</v>
       </c>
       <c r="H10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I10" t="n">
-        <v>-9.15</v>
+        <v>-7.9</v>
       </c>
       <c r="J10" t="n">
-        <v>0.298</v>
+        <v>0.259</v>
       </c>
       <c r="K10" t="n">
-        <v>2.73</v>
+        <v>2.05</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>CHECK</t>
         </is>
       </c>
     </row>
@@ -962,7 +962,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Aim 1: Minor Groove Binder</t>
+          <t>Aim 1: Minor Groove Specialist</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -986,13 +986,13 @@
         <v>2</v>
       </c>
       <c r="I11" t="n">
-        <v>-9.15</v>
+        <v>-7.5</v>
       </c>
       <c r="J11" t="n">
         <v>0.365</v>
       </c>
       <c r="K11" t="n">
-        <v>3.34</v>
+        <v>2.74</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
@@ -1008,42 +1008,42 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CHEMBL1672845</t>
+          <t>CHEMBL1683055</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Aim 1: Minor Groove Binder</t>
+          <t>Aim 1: Minor Groove Specialist</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Cc1nc2ccc(-c3nc4cc(-c5ccccc5)ccc4[nH]3)cc2[nH]1</t>
+          <t>Nc1nc2ccc(-c3ccc4nc5ccccc5nc4c3)cc2[nH]1</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>324.39</v>
+        <v>311.35</v>
       </c>
       <c r="E12" t="n">
-        <v>5.08</v>
+        <v>3.91</v>
       </c>
       <c r="F12" t="n">
-        <v>57.36</v>
+        <v>80.48</v>
       </c>
       <c r="G12" t="n">
         <v>2</v>
       </c>
       <c r="H12" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I12" t="n">
-        <v>-9.15</v>
+        <v>-7.5</v>
       </c>
       <c r="J12" t="n">
-        <v>0.308</v>
+        <v>0.482</v>
       </c>
       <c r="K12" t="n">
-        <v>2.82</v>
+        <v>3.61</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
@@ -1052,49 +1052,49 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>CHECK</t>
+          <t>PASS</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CHEMBL605817</t>
+          <t>CHEMBL1951956</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Aim 1: Minor Groove Binder</t>
+          <t>Aim 1: Minor Groove Specialist</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>c1ccc(-c2nc3cc4nc(-c5ccccc5)[nH]c4cc3[nH]2)cc1</t>
+          <t>c1ccc(-c2ccc(-c3ccc(-c4nc5ccccc5[nH]4)cc3)cc2)cc1</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>310.36</v>
+        <v>346.43</v>
       </c>
       <c r="E13" t="n">
-        <v>4.77</v>
+        <v>6.56</v>
       </c>
       <c r="F13" t="n">
-        <v>57.36</v>
+        <v>28.68</v>
       </c>
       <c r="G13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I13" t="n">
-        <v>-9.15</v>
+        <v>-7.5</v>
       </c>
       <c r="J13" t="n">
-        <v>0.322</v>
+        <v>0.289</v>
       </c>
       <c r="K13" t="n">
-        <v>2.95</v>
+        <v>2.17</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
@@ -1103,49 +1103,49 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>CHECK</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CHEMBL1962789</t>
+          <t>CHEMBL4173428</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Aim 1: Minor Groove Binder</t>
+          <t>Aim 1: Minor Groove Specialist</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Cc1ccc(-c2nc3ccc(-c4ccc5nc(=O)[nH]nc5c4)cc3[nH]2)nc1</t>
+          <t>c1ccc2[nH]c(-c3ccc(-c4nc5ccccc5[nH]4)cc3)nc2c1</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>354.37</v>
+        <v>310.36</v>
       </c>
       <c r="E14" t="n">
-        <v>3.23</v>
+        <v>4.77</v>
       </c>
       <c r="F14" t="n">
-        <v>100.21</v>
+        <v>57.36</v>
       </c>
       <c r="G14" t="n">
         <v>2</v>
       </c>
       <c r="H14" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I14" t="n">
-        <v>-9.15</v>
+        <v>-7.5</v>
       </c>
       <c r="J14" t="n">
-        <v>0.282</v>
+        <v>0.322</v>
       </c>
       <c r="K14" t="n">
-        <v>2.58</v>
+        <v>2.42</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
@@ -1161,17 +1161,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CHEMBL4173428</t>
+          <t>CHEMBL3793039</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Aim 1: Minor Groove Binder</t>
+          <t>Aim 1: Minor Groove Specialist</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>c1ccc2[nH]c(-c3ccc(-c4nc5ccccc5[nH]4)cc3)nc2c1</t>
+          <t>c1cc(-c2nc3ccccc3[nH]2)cc(-c2nc3ccccc3[nH]2)c1</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1190,13 +1190,13 @@
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>-9.15</v>
+        <v>-7.5</v>
       </c>
       <c r="J15" t="n">
         <v>0.322</v>
       </c>
       <c r="K15" t="n">
-        <v>2.95</v>
+        <v>2.42</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
@@ -1212,42 +1212,42 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CHEMBL1951976</t>
+          <t>CHEMBL174576</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Aim 1: Minor Groove Binder</t>
+          <t>Aim 1: Minor Groove Specialist</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Cc1ccc2[nH]c(-c3ccc(-c4ccc(-c5ccccc5)cc4)cc3)nc2c1</t>
+          <t>NC(=O)c1ccc2[nH]c(-c3ccc4[nH]c(-c5ccccc5)nc4c3)nc2c1</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>360.46</v>
+        <v>353.39</v>
       </c>
       <c r="E16" t="n">
-        <v>6.87</v>
+        <v>3.87</v>
       </c>
       <c r="F16" t="n">
-        <v>28.68</v>
+        <v>100.45</v>
       </c>
       <c r="G16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I16" t="n">
-        <v>-9.1</v>
+        <v>-7.5</v>
       </c>
       <c r="J16" t="n">
-        <v>0.277</v>
+        <v>0.283</v>
       </c>
       <c r="K16" t="n">
-        <v>2.52</v>
+        <v>2.12</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
@@ -1256,49 +1256,49 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>CHECK</t>
+          <t>PASS</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CHEMBL174576</t>
+          <t>CHEMBL1962789</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Aim 1: Minor Groove Binder</t>
+          <t>Aim 1: Minor Groove Specialist</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>NC(=O)c1ccc2[nH]c(-c3ccc4[nH]c(-c5ccccc5)nc4c3)nc2c1</t>
+          <t>Cc1ccc(-c2nc3ccc(-c4ccc5nc(=O)[nH]nc5c4)cc3[nH]2)nc1</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>353.39</v>
+        <v>354.37</v>
       </c>
       <c r="E17" t="n">
-        <v>3.87</v>
+        <v>3.23</v>
       </c>
       <c r="F17" t="n">
-        <v>100.45</v>
+        <v>100.21</v>
       </c>
       <c r="G17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H17" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I17" t="n">
-        <v>-9.1</v>
+        <v>-7.5</v>
       </c>
       <c r="J17" t="n">
-        <v>0.283</v>
+        <v>0.282</v>
       </c>
       <c r="K17" t="n">
-        <v>2.58</v>
+        <v>2.11</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
@@ -1314,42 +1314,42 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CHEMBL1951956</t>
+          <t>CHEMBL605817</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Aim 1: Minor Groove Binder</t>
+          <t>Aim 1: Minor Groove Specialist</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>c1ccc(-c2ccc(-c3ccc(-c4nc5ccccc5[nH]4)cc3)cc2)cc1</t>
+          <t>c1ccc(-c2nc3cc4nc(-c5ccccc5)[nH]c4cc3[nH]2)cc1</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>346.43</v>
+        <v>310.36</v>
       </c>
       <c r="E18" t="n">
-        <v>6.56</v>
+        <v>4.77</v>
       </c>
       <c r="F18" t="n">
-        <v>28.68</v>
+        <v>57.36</v>
       </c>
       <c r="G18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I18" t="n">
-        <v>-9.1</v>
+        <v>-7.5</v>
       </c>
       <c r="J18" t="n">
-        <v>0.289</v>
+        <v>0.322</v>
       </c>
       <c r="K18" t="n">
-        <v>2.63</v>
+        <v>2.42</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
@@ -1358,49 +1358,49 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>CHECK</t>
+          <t>PASS</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CHEMBL1967768</t>
+          <t>CHEMBL1672845</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Aim 1: Intercalator/Shield</t>
+          <t>Aim 1: Minor Groove Specialist</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Nc1c2ccccc2nc2c1ccc1ncccc12</t>
+          <t>Cc1nc2ccc(-c3nc4cc(-c5ccccc5)ccc4[nH]3)cc2[nH]1</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>245.28</v>
+        <v>324.39</v>
       </c>
       <c r="E19" t="n">
-        <v>3.52</v>
+        <v>5.08</v>
       </c>
       <c r="F19" t="n">
-        <v>51.8</v>
+        <v>57.36</v>
       </c>
       <c r="G19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I19" t="n">
-        <v>-8.9</v>
+        <v>-7.5</v>
       </c>
       <c r="J19" t="n">
-        <v>0.612</v>
+        <v>0.308</v>
       </c>
       <c r="K19" t="n">
-        <v>5.45</v>
+        <v>2.31</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
@@ -1409,49 +1409,49 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>CHECK</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CHEMBL5282816</t>
+          <t>CHEMBL367729</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Aim 1: Minor Groove Binder</t>
+          <t>Aim 1: Minor Groove Specialist</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>c1ccc2[nH]c(-c3ccc4n[se]nc4c3)nc2c1</t>
+          <t>N#Cc1ccc2[nH]c(-c3ccc4[nH]c(-c5ccccc5)nc4c3)nc2c1</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>299.19</v>
+        <v>335.37</v>
       </c>
       <c r="E20" t="n">
-        <v>2.23</v>
+        <v>4.64</v>
       </c>
       <c r="F20" t="n">
-        <v>54.46</v>
+        <v>81.15000000000001</v>
       </c>
       <c r="G20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H20" t="n">
         <v>3</v>
       </c>
       <c r="I20" t="n">
-        <v>-8.85</v>
+        <v>-7.5</v>
       </c>
       <c r="J20" t="n">
-        <v>0.334</v>
+        <v>0.298</v>
       </c>
       <c r="K20" t="n">
-        <v>2.96</v>
+        <v>2.23</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
@@ -1467,42 +1467,42 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CHEMBL1719169</t>
+          <t>CHEMBL1951976</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Aim 1: Intercalator/Shield</t>
+          <t>Aim 1: Minor Groove Specialist</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Nc1ccc(-c2c3ccccc3nc3ccccc23)cc1</t>
+          <t>Cc1ccc2[nH]c(-c3ccc(-c4ccc(-c5ccccc5)cc4)cc3)nc2c1</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>270.34</v>
+        <v>360.46</v>
       </c>
       <c r="E21" t="n">
-        <v>4.64</v>
+        <v>6.87</v>
       </c>
       <c r="F21" t="n">
-        <v>38.91</v>
+        <v>28.68</v>
       </c>
       <c r="G21" t="n">
         <v>1</v>
       </c>
       <c r="H21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I21" t="n">
-        <v>-8.85</v>
+        <v>-7.5</v>
       </c>
       <c r="J21" t="n">
-        <v>0.555</v>
+        <v>0.277</v>
       </c>
       <c r="K21" t="n">
-        <v>4.91</v>
+        <v>2.08</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
@@ -1511,7 +1511,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>CHECK</t>
         </is>
       </c>
     </row>
@@ -1523,7 +1523,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Aim 1: Intercalator/Shield</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1547,13 +1547,13 @@
         <v>2</v>
       </c>
       <c r="I22" t="n">
-        <v>-8.85</v>
+        <v>-7.1</v>
       </c>
       <c r="J22" t="n">
         <v>0.555</v>
       </c>
       <c r="K22" t="n">
-        <v>4.91</v>
+        <v>3.94</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
@@ -1569,42 +1569,42 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CHEMBL1413222</t>
+          <t>CHEMBL1719169</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Aim 1: Minor Groove Binder</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Cc1nc2cc(-c3nc4ccccc4[nH]3)ccc2[nH]1</t>
+          <t>Nc1ccc(-c2c3ccccc3nc3ccccc23)cc1</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>248.29</v>
+        <v>270.34</v>
       </c>
       <c r="E23" t="n">
-        <v>3.41</v>
+        <v>4.64</v>
       </c>
       <c r="F23" t="n">
-        <v>57.36</v>
+        <v>38.91</v>
       </c>
       <c r="G23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H23" t="n">
         <v>2</v>
       </c>
       <c r="I23" t="n">
-        <v>-8.85</v>
+        <v>-7.1</v>
       </c>
       <c r="J23" t="n">
-        <v>0.403</v>
+        <v>0.555</v>
       </c>
       <c r="K23" t="n">
-        <v>3.57</v>
+        <v>3.94</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
@@ -1620,42 +1620,42 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CHEMBL529603</t>
+          <t>CHEMBL1967768</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Aim 1: Minor Groove Binder</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>c1ccc(-c2ccc(-c3nc4ccccc4[nH]3)cc2)cc1</t>
+          <t>Nc1c2ccccc2nc2c1ccc1ncccc12</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>270.34</v>
+        <v>245.28</v>
       </c>
       <c r="E24" t="n">
-        <v>4.9</v>
+        <v>3.52</v>
       </c>
       <c r="F24" t="n">
-        <v>28.68</v>
+        <v>51.8</v>
       </c>
       <c r="G24" t="n">
         <v>1</v>
       </c>
       <c r="H24" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I24" t="n">
-        <v>-8.800000000000001</v>
+        <v>-7.1</v>
       </c>
       <c r="J24" t="n">
-        <v>0.37</v>
+        <v>0.612</v>
       </c>
       <c r="K24" t="n">
-        <v>3.26</v>
+        <v>4.35</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
@@ -1671,7 +1671,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CHEMBL1927181</t>
+          <t>CHEMBL4087126</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1681,17 +1681,17 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Cc1ccc(C(=O)Nc2nc3ccc(-c4ccc5nc6ccccc6nc5c4)cc3[nH]2)cc1</t>
+          <t>O=c1cc(-c2ccc(-c3ccccc3)cc2)oc2cc(O)cc(O)c12</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>429.48</v>
+        <v>330.34</v>
       </c>
       <c r="E25" t="n">
-        <v>5.89</v>
+        <v>4.54</v>
       </c>
       <c r="F25" t="n">
-        <v>83.56</v>
+        <v>70.67</v>
       </c>
       <c r="G25" t="n">
         <v>2</v>
@@ -1700,13 +1700,13 @@
         <v>4</v>
       </c>
       <c r="I25" t="n">
-        <v>-8.65</v>
+        <v>-7.1</v>
       </c>
       <c r="J25" t="n">
-        <v>0.233</v>
+        <v>1.816</v>
       </c>
       <c r="K25" t="n">
-        <v>2.02</v>
+        <v>12.89</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
@@ -1715,49 +1715,49 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>CHECK</t>
+          <t>PASS</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CHEMBL357429</t>
+          <t>CHEMBL529603</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Aim 1: Intercalator/Shield</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Cc1ccc2nc3ccccc3c(N)c2c1</t>
+          <t>c1ccc(-c2ccc(-c3nc4ccccc4[nH]3)cc2)cc1</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>208.26</v>
+        <v>270.34</v>
       </c>
       <c r="E26" t="n">
-        <v>3.28</v>
+        <v>4.9</v>
       </c>
       <c r="F26" t="n">
-        <v>38.91</v>
+        <v>28.68</v>
       </c>
       <c r="G26" t="n">
         <v>1</v>
       </c>
       <c r="H26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I26" t="n">
-        <v>-8.550000000000001</v>
+        <v>-7.1</v>
       </c>
       <c r="J26" t="n">
-        <v>0.72</v>
+        <v>0.37</v>
       </c>
       <c r="K26" t="n">
-        <v>6.16</v>
+        <v>2.63</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
@@ -1773,42 +1773,42 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CHEMBL1741616</t>
+          <t>CHEMBL5282816</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Aim 1: Intercalator/Shield</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Nc1c2ccccc2nc2c(O)cccc12</t>
+          <t>c1ccc2[nH]c(-c3ccc4n[se]nc4c3)nc2c1</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>210.24</v>
+        <v>299.19</v>
       </c>
       <c r="E27" t="n">
-        <v>2.68</v>
+        <v>2.23</v>
       </c>
       <c r="F27" t="n">
-        <v>59.14</v>
+        <v>54.46</v>
       </c>
       <c r="G27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H27" t="n">
         <v>3</v>
       </c>
       <c r="I27" t="n">
-        <v>-8.550000000000001</v>
+        <v>-7.1</v>
       </c>
       <c r="J27" t="n">
-        <v>2.14</v>
+        <v>0.334</v>
       </c>
       <c r="K27" t="n">
-        <v>18.3</v>
+        <v>2.37</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
@@ -1824,42 +1824,42 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CHEMBL148785</t>
+          <t>CHEMBL1413222</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Aim 1: Intercalator/Shield</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Nc1c2ccccc2nc2c(Cl)cccc12</t>
+          <t>Cc1nc2cc(-c3nc4ccccc4[nH]3)ccc2[nH]1</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>228.68</v>
+        <v>248.29</v>
       </c>
       <c r="E28" t="n">
-        <v>3.62</v>
+        <v>3.41</v>
       </c>
       <c r="F28" t="n">
-        <v>38.91</v>
+        <v>57.36</v>
       </c>
       <c r="G28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H28" t="n">
         <v>2</v>
       </c>
       <c r="I28" t="n">
-        <v>-8.550000000000001</v>
+        <v>-7.1</v>
       </c>
       <c r="J28" t="n">
-        <v>0.656</v>
+        <v>0.403</v>
       </c>
       <c r="K28" t="n">
-        <v>5.61</v>
+        <v>2.86</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
@@ -1875,42 +1875,42 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CHEMBL343190</t>
+          <t>CHEMBL5431952</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Aim 1: Intercalator/Shield</t>
+          <t>Aim 3: Dual-Action Lead</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Cc1cccc2c(N)c3ccccc3nc12</t>
+          <t>O=c1cc(-c2cccc(-c3ccc(O)cc3)c2)oc2cc(O)cc(O)c12</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>208.26</v>
+        <v>346.34</v>
       </c>
       <c r="E29" t="n">
-        <v>3.28</v>
+        <v>4.24</v>
       </c>
       <c r="F29" t="n">
-        <v>38.91</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="G29" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H29" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I29" t="n">
-        <v>-8.550000000000001</v>
+        <v>-7.1</v>
       </c>
       <c r="J29" t="n">
-        <v>0.72</v>
+        <v>2.599</v>
       </c>
       <c r="K29" t="n">
-        <v>6.16</v>
+        <v>18.45</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
@@ -1926,42 +1926,42 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CHEMBL147657</t>
+          <t>CHEMBL183745</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Aim 1: Intercalator/Shield</t>
+          <t>Aim 2: ROS Scavenger Specialist</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Nc1c2ccccc2nc2ccc(Cl)cc12</t>
+          <t>COc1cc(O)c2c(=O)cc(-c3ccc(O)c(O)c3)oc2c1</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>228.68</v>
+        <v>300.27</v>
       </c>
       <c r="E30" t="n">
-        <v>3.62</v>
+        <v>2.59</v>
       </c>
       <c r="F30" t="n">
-        <v>38.91</v>
+        <v>100.13</v>
       </c>
       <c r="G30" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H30" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="I30" t="n">
-        <v>-8.550000000000001</v>
+        <v>-6.7</v>
       </c>
       <c r="J30" t="n">
-        <v>0.656</v>
+        <v>2.997</v>
       </c>
       <c r="K30" t="n">
-        <v>5.61</v>
+        <v>20.08</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
@@ -1977,42 +1977,42 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CHEMBL548175</t>
+          <t>CHEMBL457821</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Aim 1: Intercalator/Shield</t>
+          <t>Aim 2: ROS Scavenger Specialist</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Cl.Nc1ccc2c(N)c3ccccc3nc2c1</t>
+          <t>O=c1cc(-c2cccc(O)c2)oc2cc(O)cc(O)c12</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>245.71</v>
+        <v>270.24</v>
       </c>
       <c r="E31" t="n">
-        <v>2.97</v>
+        <v>2.58</v>
       </c>
       <c r="F31" t="n">
-        <v>64.93000000000001</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="G31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H31" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I31" t="n">
-        <v>-8.550000000000001</v>
+        <v>-6.7</v>
       </c>
       <c r="J31" t="n">
-        <v>1.221</v>
+        <v>3.33</v>
       </c>
       <c r="K31" t="n">
-        <v>10.44</v>
+        <v>22.31</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
@@ -2028,42 +2028,42 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CHEMBL148238</t>
+          <t>CHEMBL28</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Aim 1: Intercalator/Shield</t>
+          <t>Aim 2: ROS Scavenger Specialist</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Cc1ccc2c(N)c3ccccc3nc2c1</t>
+          <t>O=c1cc(-c2ccc(O)cc2)oc2cc(O)cc(O)c12</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>208.26</v>
+        <v>270.24</v>
       </c>
       <c r="E32" t="n">
-        <v>3.28</v>
+        <v>2.58</v>
       </c>
       <c r="F32" t="n">
-        <v>38.91</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="G32" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H32" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I32" t="n">
-        <v>-8.550000000000001</v>
+        <v>-6.7</v>
       </c>
       <c r="J32" t="n">
-        <v>0.72</v>
+        <v>3.33</v>
       </c>
       <c r="K32" t="n">
-        <v>6.16</v>
+        <v>22.31</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
@@ -2079,42 +2079,42 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CHEMBL147630</t>
+          <t>CHEMBL5418159</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Aim 1: Intercalator/Shield</t>
+          <t>Aim 2: ROS Scavenger Specialist</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Nc1ccc2c(N)c3ccccc3nc2c1</t>
+          <t>O=c1cc(-c2ccc(O)c(O)c2)oc2cc(F)cc(O)c12</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>209.25</v>
+        <v>288.23</v>
       </c>
       <c r="E33" t="n">
-        <v>2.55</v>
+        <v>2.72</v>
       </c>
       <c r="F33" t="n">
-        <v>64.93000000000001</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="G33" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H33" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I33" t="n">
-        <v>-8.550000000000001</v>
+        <v>-6.7</v>
       </c>
       <c r="J33" t="n">
-        <v>1.434</v>
+        <v>3.123</v>
       </c>
       <c r="K33" t="n">
-        <v>12.26</v>
+        <v>20.92</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
@@ -2130,42 +2130,42 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CHEMBL1883643</t>
+          <t>CHEMBL528704</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Aim 1: Intercalator/Shield</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Cc1c2ccccc2nc2ccccc12</t>
+          <t>Nc1c2ccccc2nc2cc([N+](=O)[O-])ccc12</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>193.25</v>
+        <v>239.23</v>
       </c>
       <c r="E34" t="n">
-        <v>3.7</v>
+        <v>2.88</v>
       </c>
       <c r="F34" t="n">
-        <v>12.89</v>
+        <v>82.05</v>
       </c>
       <c r="G34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H34" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I34" t="n">
-        <v>-8.550000000000001</v>
+        <v>-6.7</v>
       </c>
       <c r="J34" t="n">
-        <v>0.517</v>
+        <v>0.627</v>
       </c>
       <c r="K34" t="n">
-        <v>4.42</v>
+        <v>4.2</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
@@ -2181,24 +2181,24 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CHEMBL581508</t>
+          <t>CHEMBL1330022</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Aim 1: Intercalator/Shield</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Nc1c2ccccc2nc2cc(C(F)(F)F)ccc12</t>
+          <t>Cl.Nc1c2ccccc2nc2ccccc12</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>262.23</v>
+        <v>230.7</v>
       </c>
       <c r="E35" t="n">
-        <v>3.99</v>
+        <v>3.39</v>
       </c>
       <c r="F35" t="n">
         <v>38.91</v>
@@ -2210,13 +2210,13 @@
         <v>2</v>
       </c>
       <c r="I35" t="n">
-        <v>-8.550000000000001</v>
+        <v>-6.7</v>
       </c>
       <c r="J35" t="n">
-        <v>0.572</v>
+        <v>0.65</v>
       </c>
       <c r="K35" t="n">
-        <v>4.89</v>
+        <v>4.36</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
@@ -2232,42 +2232,42 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CHEMBL2180144</t>
+          <t>CHEMBL171045</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Aim 1: Intercalator/Shield</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Clc1c2ccccc2nc2ccccc12</t>
+          <t>Nc1cccc2nc3ccccc3c(N)c12</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>213.67</v>
+        <v>209.25</v>
       </c>
       <c r="E36" t="n">
-        <v>4.04</v>
+        <v>2.55</v>
       </c>
       <c r="F36" t="n">
-        <v>12.89</v>
+        <v>64.93000000000001</v>
       </c>
       <c r="G36" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H36" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I36" t="n">
-        <v>-8.550000000000001</v>
+        <v>-6.7</v>
       </c>
       <c r="J36" t="n">
-        <v>0.468</v>
+        <v>1.434</v>
       </c>
       <c r="K36" t="n">
-        <v>4</v>
+        <v>9.609999999999999</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
@@ -2283,42 +2283,42 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CHEMBL3290780</t>
+          <t>CHEMBL2396656</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Aim 1: Intercalator/Shield</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Nc1nc2ccccc2c2ccccc12</t>
+          <t>Oc1ccc2[nH]c(-c3ccccc3)nc2c1</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>194.24</v>
+        <v>210.24</v>
       </c>
       <c r="E37" t="n">
-        <v>2.97</v>
+        <v>2.94</v>
       </c>
       <c r="F37" t="n">
-        <v>38.91</v>
+        <v>48.91</v>
       </c>
       <c r="G37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H37" t="n">
         <v>2</v>
       </c>
       <c r="I37" t="n">
-        <v>-8.550000000000001</v>
+        <v>-6.7</v>
       </c>
       <c r="J37" t="n">
-        <v>0.772</v>
+        <v>1.427</v>
       </c>
       <c r="K37" t="n">
-        <v>6.6</v>
+        <v>9.56</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
@@ -2339,7 +2339,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Aim 1: Intercalator/Shield</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2363,13 +2363,13 @@
         <v>4</v>
       </c>
       <c r="I38" t="n">
-        <v>-8.550000000000001</v>
+        <v>-6.7</v>
       </c>
       <c r="J38" t="n">
         <v>0.764</v>
       </c>
       <c r="K38" t="n">
-        <v>6.53</v>
+        <v>5.12</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -2385,24 +2385,24 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CHEMBL171045</t>
+          <t>CHEMBL548175</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Aim 1: Intercalator/Shield</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Nc1cccc2nc3ccccc3c(N)c12</t>
+          <t>Cl.Nc1ccc2c(N)c3ccccc3nc2c1</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>209.25</v>
+        <v>245.71</v>
       </c>
       <c r="E39" t="n">
-        <v>2.55</v>
+        <v>2.97</v>
       </c>
       <c r="F39" t="n">
         <v>64.93000000000001</v>
@@ -2414,13 +2414,13 @@
         <v>3</v>
       </c>
       <c r="I39" t="n">
-        <v>-8.550000000000001</v>
+        <v>-6.7</v>
       </c>
       <c r="J39" t="n">
-        <v>1.434</v>
+        <v>1.221</v>
       </c>
       <c r="K39" t="n">
-        <v>12.26</v>
+        <v>8.18</v>
       </c>
       <c r="L39" t="inlineStr">
         <is>
@@ -2436,24 +2436,24 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CHEMBL146512</t>
+          <t>CHEMBL3290780</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Aim 1: Intercalator/Shield</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Nc1c2ccccc2nc2cc(Cl)ccc12</t>
+          <t>Nc1nc2ccccc2c2ccccc12</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>228.68</v>
+        <v>194.24</v>
       </c>
       <c r="E40" t="n">
-        <v>3.62</v>
+        <v>2.97</v>
       </c>
       <c r="F40" t="n">
         <v>38.91</v>
@@ -2465,13 +2465,13 @@
         <v>2</v>
       </c>
       <c r="I40" t="n">
-        <v>-8.550000000000001</v>
+        <v>-6.7</v>
       </c>
       <c r="J40" t="n">
-        <v>0.656</v>
+        <v>0.772</v>
       </c>
       <c r="K40" t="n">
-        <v>5.61</v>
+        <v>5.17</v>
       </c>
       <c r="L40" t="inlineStr">
         <is>
@@ -2487,42 +2487,42 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CHEMBL43184</t>
+          <t>CHEMBL4547449</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Aim 1: Intercalator/Shield</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Nc1c2ccccc2nc2ccccc12</t>
+          <t>Br.Oc1ccc2[nH]c(-c3ccccc3)nc2c1</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>194.24</v>
+        <v>291.15</v>
       </c>
       <c r="E41" t="n">
-        <v>2.97</v>
+        <v>3.51</v>
       </c>
       <c r="F41" t="n">
-        <v>38.91</v>
+        <v>48.91</v>
       </c>
       <c r="G41" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H41" t="n">
         <v>2</v>
       </c>
       <c r="I41" t="n">
-        <v>-8.550000000000001</v>
+        <v>-6.7</v>
       </c>
       <c r="J41" t="n">
-        <v>0.772</v>
+        <v>1.03</v>
       </c>
       <c r="K41" t="n">
-        <v>6.6</v>
+        <v>6.9</v>
       </c>
       <c r="L41" t="inlineStr">
         <is>
@@ -2538,27 +2538,27 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CHEMBL1308088</t>
+          <t>CHEMBL148238</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Aim 1: Intercalator/Shield</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Cl.Nc1c2ccccc2nc2ccccc12.O</t>
+          <t>Cc1ccc2c(N)c3ccccc3nc2c1</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>248.71</v>
+        <v>208.26</v>
       </c>
       <c r="E42" t="n">
-        <v>2.57</v>
+        <v>3.28</v>
       </c>
       <c r="F42" t="n">
-        <v>70.41</v>
+        <v>38.91</v>
       </c>
       <c r="G42" t="n">
         <v>1</v>
@@ -2567,13 +2567,13 @@
         <v>2</v>
       </c>
       <c r="I42" t="n">
-        <v>-8.550000000000001</v>
+        <v>-6.7</v>
       </c>
       <c r="J42" t="n">
-        <v>0.603</v>
+        <v>0.72</v>
       </c>
       <c r="K42" t="n">
-        <v>5.16</v>
+        <v>4.82</v>
       </c>
       <c r="L42" t="inlineStr">
         <is>
@@ -2589,42 +2589,42 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CHEMBL1330022</t>
+          <t>CHEMBL1330989</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Aim 1: Intercalator/Shield</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Cl.Nc1c2ccccc2nc2ccccc12</t>
+          <t>Nc1ccc2[nH]c(-c3ccccc3)nc2c1</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>230.7</v>
+        <v>209.25</v>
       </c>
       <c r="E43" t="n">
-        <v>3.39</v>
+        <v>2.81</v>
       </c>
       <c r="F43" t="n">
-        <v>38.91</v>
+        <v>54.7</v>
       </c>
       <c r="G43" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H43" t="n">
         <v>2</v>
       </c>
       <c r="I43" t="n">
-        <v>-8.550000000000001</v>
+        <v>-6.7</v>
       </c>
       <c r="J43" t="n">
-        <v>0.65</v>
+        <v>0.717</v>
       </c>
       <c r="K43" t="n">
-        <v>5.56</v>
+        <v>4.8</v>
       </c>
       <c r="L43" t="inlineStr">
         <is>
@@ -2640,42 +2640,42 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CHEMBL1596095</t>
+          <t>CHEMBL148785</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Aim 1: Minor Groove Binder</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Fc1ccc(-c2nc3ccccc3[nH]2)cc1</t>
+          <t>Nc1c2ccccc2nc2c(Cl)cccc12</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>212.23</v>
+        <v>228.68</v>
       </c>
       <c r="E44" t="n">
-        <v>3.37</v>
+        <v>3.62</v>
       </c>
       <c r="F44" t="n">
-        <v>28.68</v>
+        <v>38.91</v>
       </c>
       <c r="G44" t="n">
         <v>1</v>
       </c>
       <c r="H44" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I44" t="n">
-        <v>-8.5</v>
+        <v>-6.7</v>
       </c>
       <c r="J44" t="n">
-        <v>0.471</v>
+        <v>0.656</v>
       </c>
       <c r="K44" t="n">
-        <v>4</v>
+        <v>4.4</v>
       </c>
       <c r="L44" t="inlineStr">
         <is>
@@ -2691,42 +2691,42 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CHEMBL2283280</t>
+          <t>CHEMBL578723</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Aim 1: Minor Groove Binder</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Cc1ccc(-c2nc3ccccc3[nH]2)cc1</t>
+          <t>COc1ccc2nc3ccccc3c(N)c2c1</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>208.26</v>
+        <v>224.26</v>
       </c>
       <c r="E45" t="n">
-        <v>3.54</v>
+        <v>2.98</v>
       </c>
       <c r="F45" t="n">
-        <v>28.68</v>
+        <v>48.14</v>
       </c>
       <c r="G45" t="n">
         <v>1</v>
       </c>
       <c r="H45" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I45" t="n">
-        <v>-8.5</v>
+        <v>-6.7</v>
       </c>
       <c r="J45" t="n">
-        <v>0.48</v>
+        <v>0.669</v>
       </c>
       <c r="K45" t="n">
-        <v>4.08</v>
+        <v>4.48</v>
       </c>
       <c r="L45" t="inlineStr">
         <is>
@@ -2742,42 +2742,42 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CHEMBL4547449</t>
+          <t>CHEMBL3896909</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Aim 1: Minor Groove Binder</t>
+          <t>Aim 2: ROS Scavenger Specialist</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Br.Oc1ccc2[nH]c(-c3ccccc3)nc2c1</t>
+          <t>Oc1cc(O)c2c(=S)cc(-c3ccc(O)c(O)c3)oc2c1</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>291.15</v>
+        <v>302.31</v>
       </c>
       <c r="E46" t="n">
-        <v>3.51</v>
+        <v>3.65</v>
       </c>
       <c r="F46" t="n">
-        <v>48.91</v>
+        <v>94.06</v>
       </c>
       <c r="G46" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H46" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="I46" t="n">
-        <v>-8.5</v>
+        <v>-6.7</v>
       </c>
       <c r="J46" t="n">
-        <v>1.03</v>
+        <v>3.969</v>
       </c>
       <c r="K46" t="n">
-        <v>8.76</v>
+        <v>26.59</v>
       </c>
       <c r="L46" t="inlineStr">
         <is>
@@ -2793,42 +2793,42 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CHEMBL2396656</t>
+          <t>CHEMBL151</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Aim 1: Minor Groove Binder</t>
+          <t>Aim 2: ROS Scavenger Specialist</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Oc1ccc2[nH]c(-c3ccccc3)nc2c1</t>
+          <t>O=c1cc(-c2ccc(O)c(O)c2)oc2cc(O)cc(O)c12</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>210.24</v>
+        <v>286.24</v>
       </c>
       <c r="E47" t="n">
-        <v>2.94</v>
+        <v>2.28</v>
       </c>
       <c r="F47" t="n">
-        <v>48.91</v>
+        <v>111.13</v>
       </c>
       <c r="G47" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H47" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="I47" t="n">
-        <v>-8.5</v>
+        <v>-6.7</v>
       </c>
       <c r="J47" t="n">
-        <v>1.427</v>
+        <v>4.192</v>
       </c>
       <c r="K47" t="n">
-        <v>12.13</v>
+        <v>28.09</v>
       </c>
       <c r="L47" t="inlineStr">
         <is>
@@ -2844,42 +2844,42 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CHEMBL1534413</t>
+          <t>CHEMBL511458</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Aim 1: Minor Groove Binder</t>
+          <t>Aim 2: ROS Scavenger Specialist</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Clc1ccc2[nH]c(-c3ccccc3)nc2c1</t>
+          <t>Oc1cc(O)c2c(c1)oc(-c1cc(O)c(O)c(O)c1)c(O)c2=O</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>228.68</v>
+        <v>318.24</v>
       </c>
       <c r="E48" t="n">
-        <v>3.88</v>
+        <v>1.69</v>
       </c>
       <c r="F48" t="n">
-        <v>28.68</v>
+        <v>151.59</v>
       </c>
       <c r="G48" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H48" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="I48" t="n">
-        <v>-8.5</v>
+        <v>-6.7</v>
       </c>
       <c r="J48" t="n">
-        <v>0.437</v>
+        <v>5.656</v>
       </c>
       <c r="K48" t="n">
-        <v>3.71</v>
+        <v>37.9</v>
       </c>
       <c r="L48" t="inlineStr">
         <is>
@@ -2895,42 +2895,42 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CHEMBL153535</t>
+          <t>CHEMBL247484</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Aim 1: Minor Groove Binder</t>
+          <t>Aim 2: ROS Scavenger Specialist</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>c1ccc(-c2nc3ccccc3[nH]2)cc1</t>
+          <t>O=c1cc(-c2cc(O)c(O)c(O)c2)oc2cc(O)cc(O)c12</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>194.24</v>
+        <v>302.24</v>
       </c>
       <c r="E49" t="n">
-        <v>3.23</v>
+        <v>1.99</v>
       </c>
       <c r="F49" t="n">
-        <v>28.68</v>
+        <v>131.36</v>
       </c>
       <c r="G49" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H49" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I49" t="n">
-        <v>-8.5</v>
+        <v>-6.7</v>
       </c>
       <c r="J49" t="n">
-        <v>0.515</v>
+        <v>4.963</v>
       </c>
       <c r="K49" t="n">
-        <v>4.38</v>
+        <v>33.25</v>
       </c>
       <c r="L49" t="inlineStr">
         <is>
@@ -2946,42 +2946,42 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CHEMBL531708</t>
+          <t>CHEMBL264037</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Aim 1: Intercalator/Shield</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Cl.Nc1c2ccccc2nc2cc([N+](=O)[O-])ccc12</t>
+          <t>O=c1cc(-c2ccc(Cl)cc2)oc2cc(O)cc(O)c12</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>275.69</v>
+        <v>288.69</v>
       </c>
       <c r="E50" t="n">
-        <v>3.3</v>
+        <v>3.52</v>
       </c>
       <c r="F50" t="n">
-        <v>82.05</v>
+        <v>70.67</v>
       </c>
       <c r="G50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H50" t="n">
         <v>4</v>
       </c>
       <c r="I50" t="n">
-        <v>-8.5</v>
+        <v>-6.7</v>
       </c>
       <c r="J50" t="n">
-        <v>0.544</v>
+        <v>2.078</v>
       </c>
       <c r="K50" t="n">
-        <v>4.62</v>
+        <v>13.92</v>
       </c>
       <c r="L50" t="inlineStr">
         <is>
@@ -2997,42 +2997,42 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CHEMBL1330989</t>
+          <t>CHEMBL214321</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Aim 1: Minor Groove Binder</t>
+          <t>Aim 2: ROS Scavenger Specialist</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Nc1ccc2[nH]c(-c3ccccc3)nc2c1</t>
+          <t>COc1cc(-c2cc(=O)c3c(O)cc(O)cc3o2)ccc1O</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>209.25</v>
+        <v>300.27</v>
       </c>
       <c r="E51" t="n">
-        <v>2.81</v>
+        <v>2.59</v>
       </c>
       <c r="F51" t="n">
-        <v>54.7</v>
+        <v>100.13</v>
       </c>
       <c r="G51" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H51" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="I51" t="n">
-        <v>-8.5</v>
+        <v>-6.7</v>
       </c>
       <c r="J51" t="n">
-        <v>0.717</v>
+        <v>2.997</v>
       </c>
       <c r="K51" t="n">
-        <v>6.09</v>
+        <v>20.08</v>
       </c>
       <c r="L51" t="inlineStr">
         <is>
@@ -3048,42 +3048,42 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CHEMBL578723</t>
+          <t>CHEMBL167154</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Aim 1: Intercalator/Shield</t>
+          <t>Aim 2: ROS Scavenger Specialist</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>COc1ccc2nc3ccccc3c(N)c2c1</t>
+          <t>Nc1ccc(-c2cc(=O)c3c(O)cc(O)cc3o2)cc1</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>224.26</v>
+        <v>269.26</v>
       </c>
       <c r="E52" t="n">
-        <v>2.98</v>
+        <v>2.45</v>
       </c>
       <c r="F52" t="n">
-        <v>48.14</v>
+        <v>96.69</v>
       </c>
       <c r="G52" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H52" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I52" t="n">
-        <v>-8.5</v>
+        <v>-6.7</v>
       </c>
       <c r="J52" t="n">
-        <v>0.669</v>
+        <v>2.785</v>
       </c>
       <c r="K52" t="n">
-        <v>5.69</v>
+        <v>18.66</v>
       </c>
       <c r="L52" t="inlineStr">
         <is>
@@ -3099,42 +3099,42 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CHEMBL528704</t>
+          <t>CHEMBL5398631</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Aim 1: Intercalator/Shield</t>
+          <t>Aim 2: ROS Scavenger Specialist</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Nc1c2ccccc2nc2cc([N+](=O)[O-])ccc12</t>
+          <t>O=C(O)c1cc(-c2cc(=O)c3c(O)cc(O)cc3o2)ccc1O</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>239.23</v>
+        <v>314.25</v>
       </c>
       <c r="E53" t="n">
-        <v>2.88</v>
+        <v>2.27</v>
       </c>
       <c r="F53" t="n">
-        <v>82.05</v>
+        <v>128.2</v>
       </c>
       <c r="G53" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H53" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I53" t="n">
-        <v>-8.5</v>
+        <v>-6.7</v>
       </c>
       <c r="J53" t="n">
-        <v>0.627</v>
+        <v>2.864</v>
       </c>
       <c r="K53" t="n">
-        <v>5.33</v>
+        <v>19.19</v>
       </c>
       <c r="L53" t="inlineStr">
         <is>
@@ -3150,42 +3150,42 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CHEMBL176543</t>
+          <t>CHEMBL182262</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Aim 1: Intercalator/Shield</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>CCN(CC)CCNc1c2ccccc2nc2ccccc12</t>
+          <t>Cc1ccc(-c2cc(=O)c3c(O)cc(O)cc3o2)cc1</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>293.41</v>
+        <v>268.27</v>
       </c>
       <c r="E54" t="n">
-        <v>4.14</v>
+        <v>3.18</v>
       </c>
       <c r="F54" t="n">
-        <v>28.16</v>
+        <v>70.67</v>
       </c>
       <c r="G54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H54" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I54" t="n">
-        <v>-8.25</v>
+        <v>-6.7</v>
       </c>
       <c r="J54" t="n">
-        <v>0.341</v>
+        <v>2.237</v>
       </c>
       <c r="K54" t="n">
-        <v>2.81</v>
+        <v>14.99</v>
       </c>
       <c r="L54" t="inlineStr">
         <is>
@@ -3201,27 +3201,27 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CHEMBL268354</t>
+          <t>CHEMBL486407</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Aim 1: Intercalator/Shield</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Nc1nc(N)c2ccccc2n1</t>
+          <t>O=c1cc(-c2ccc(F)cc2)oc2cc(O)cc(O)c12</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>160.18</v>
+        <v>272.23</v>
       </c>
       <c r="E55" t="n">
-        <v>0.79</v>
+        <v>3.01</v>
       </c>
       <c r="F55" t="n">
-        <v>77.81999999999999</v>
+        <v>70.67</v>
       </c>
       <c r="G55" t="n">
         <v>2</v>
@@ -3230,13 +3230,13 @@
         <v>4</v>
       </c>
       <c r="I55" t="n">
-        <v>-8.199999999999999</v>
+        <v>-6.7</v>
       </c>
       <c r="J55" t="n">
-        <v>1.873</v>
+        <v>2.204</v>
       </c>
       <c r="K55" t="n">
-        <v>15.36</v>
+        <v>14.77</v>
       </c>
       <c r="L55" t="inlineStr">
         <is>
@@ -3245,155 +3245,155 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>CHECK</t>
+          <t>PASS</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CHEMBL1779470</t>
+          <t>CHEMBL1741616</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Aim 2: Flavonoid Scavenger</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>O=c1cc(-c2ccc(O)c(-c3cc(-c4cc(=O)c5c(O)cc(O)cc5o4)ccc3O)c2)oc2cc(O)cc(O)c12</t>
+          <t>Nc1c2ccccc2nc2c(O)cccc12</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>538.46</v>
+        <v>210.24</v>
       </c>
       <c r="E56" t="n">
-        <v>5.13</v>
+        <v>2.68</v>
       </c>
       <c r="F56" t="n">
-        <v>181.8</v>
+        <v>59.14</v>
       </c>
       <c r="G56" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H56" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="I56" t="n">
-        <v>-6.55</v>
+        <v>-6.7</v>
       </c>
       <c r="J56" t="n">
-        <v>3.343</v>
+        <v>2.14</v>
       </c>
       <c r="K56" t="n">
-        <v>21.9</v>
+        <v>14.34</v>
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>CHECK</t>
+          <t>PASS</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CHEMBL4847220</t>
+          <t>CHEMBL117</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Aim 2: Flavonoid Scavenger</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>O=c1cc(-c2cccc(-c3c(O)cc(O)c4c(=O)cc(-c5ccc(O)c(O)c5)oc34)c2)oc2cc(O)cc(O)c12</t>
+          <t>O=c1cc(-c2ccccc2)oc2cc(O)cc(O)c12</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>538.46</v>
+        <v>254.24</v>
       </c>
       <c r="E57" t="n">
-        <v>5.13</v>
+        <v>2.87</v>
       </c>
       <c r="F57" t="n">
-        <v>181.8</v>
+        <v>70.67</v>
       </c>
       <c r="G57" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H57" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="I57" t="n">
-        <v>-6.55</v>
+        <v>-6.7</v>
       </c>
       <c r="J57" t="n">
-        <v>3.343</v>
+        <v>2.36</v>
       </c>
       <c r="K57" t="n">
-        <v>21.9</v>
+        <v>15.81</v>
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>CHECK</t>
+          <t>PASS</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CHEMBL1990497</t>
+          <t>CHEMBL147630</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Aim 2: Flavonoid Scavenger</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>O=c1cc(-c2cc(O)c(O)c(-c3c(O)cc4oc(-c5ccc(O)c(O)c5)cc(=O)c4c3O)c2)oc2cc(O)cc(O)c12</t>
+          <t>Nc1ccc2c(N)c3ccccc3nc2c1</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>570.46</v>
+        <v>209.25</v>
       </c>
       <c r="E58" t="n">
-        <v>4.55</v>
+        <v>2.55</v>
       </c>
       <c r="F58" t="n">
-        <v>222.26</v>
+        <v>64.93000000000001</v>
       </c>
       <c r="G58" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="H58" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="I58" t="n">
-        <v>-6.55</v>
+        <v>-6.7</v>
       </c>
       <c r="J58" t="n">
-        <v>4.207</v>
+        <v>1.434</v>
       </c>
       <c r="K58" t="n">
-        <v>27.56</v>
+        <v>9.609999999999999</v>
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
@@ -3405,42 +3405,42 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CHEMBL5431952</t>
+          <t>CHEMBL1821732</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Aim 2: Flavonoid Scavenger</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>O=c1cc(-c2cccc(-c3ccc(O)cc3)c2)oc2cc(O)cc(O)c12</t>
+          <t>O=c1cc(-c2ccc(F)c(F)c2)oc2cc(O)cc(O)c12</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>346.34</v>
+        <v>290.22</v>
       </c>
       <c r="E59" t="n">
-        <v>4.24</v>
+        <v>3.15</v>
       </c>
       <c r="F59" t="n">
-        <v>90.90000000000001</v>
+        <v>70.67</v>
       </c>
       <c r="G59" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H59" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I59" t="n">
-        <v>-6.2</v>
+        <v>-6.7</v>
       </c>
       <c r="J59" t="n">
-        <v>2.599</v>
+        <v>2.067</v>
       </c>
       <c r="K59" t="n">
-        <v>16.11</v>
+        <v>13.85</v>
       </c>
       <c r="L59" t="inlineStr">
         <is>
@@ -3456,24 +3456,24 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CHEMBL4087126</t>
+          <t>CHEMBL471181</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Aim 2: Flavonoid Scavenger</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>O=c1cc(-c2ccc(-c3ccccc3)cc2)oc2cc(O)cc(O)c12</t>
+          <t>O=c1cc(-c2ccc(Br)cc2)oc2cc(O)cc(O)c12</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>330.34</v>
+        <v>333.14</v>
       </c>
       <c r="E60" t="n">
-        <v>4.54</v>
+        <v>3.63</v>
       </c>
       <c r="F60" t="n">
         <v>70.67</v>
@@ -3485,13 +3485,13 @@
         <v>4</v>
       </c>
       <c r="I60" t="n">
-        <v>-6.2</v>
+        <v>-6.7</v>
       </c>
       <c r="J60" t="n">
-        <v>1.816</v>
+        <v>1.801</v>
       </c>
       <c r="K60" t="n">
-        <v>11.26</v>
+        <v>12.07</v>
       </c>
       <c r="L60" t="inlineStr">
         <is>
@@ -3507,24 +3507,24 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CHEMBL182262</t>
+          <t>CHEMBL1822222</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Aim 2: Flavonoid Scavenger</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Cc1ccc(-c2cc(=O)c3c(O)cc(O)cc3o2)cc1</t>
+          <t>O=c1cc(-c2ccc(I)cc2)oc2cc(O)cc(O)c12</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>268.27</v>
+        <v>380.14</v>
       </c>
       <c r="E61" t="n">
-        <v>3.18</v>
+        <v>3.48</v>
       </c>
       <c r="F61" t="n">
         <v>70.67</v>
@@ -3536,13 +3536,13 @@
         <v>4</v>
       </c>
       <c r="I61" t="n">
-        <v>-6.05</v>
+        <v>-6.7</v>
       </c>
       <c r="J61" t="n">
-        <v>2.237</v>
+        <v>1.578</v>
       </c>
       <c r="K61" t="n">
-        <v>13.53</v>
+        <v>10.57</v>
       </c>
       <c r="L61" t="inlineStr">
         <is>
@@ -3558,42 +3558,42 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CHEMBL28</t>
+          <t>CHEMBL1277701</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Aim 2: Flavonoid Scavenger</t>
+          <t>Aim 2: ROS Scavenger Specialist</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>O=c1cc(-c2ccc(O)cc2)oc2cc(O)cc(O)c12</t>
+          <t>COc1cc(O)cc2oc(-c3ccc(O)c(O)c3)cc(=O)c12</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>270.24</v>
+        <v>300.27</v>
       </c>
       <c r="E62" t="n">
-        <v>2.58</v>
+        <v>2.59</v>
       </c>
       <c r="F62" t="n">
-        <v>90.90000000000001</v>
+        <v>100.13</v>
       </c>
       <c r="G62" t="n">
         <v>3</v>
       </c>
       <c r="H62" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I62" t="n">
-        <v>-6.05</v>
+        <v>-6.7</v>
       </c>
       <c r="J62" t="n">
-        <v>3.33</v>
+        <v>2.997</v>
       </c>
       <c r="K62" t="n">
-        <v>20.15</v>
+        <v>20.08</v>
       </c>
       <c r="L62" t="inlineStr">
         <is>
@@ -3609,42 +3609,42 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CHEMBL5418159</t>
+          <t>CHEMBL90568</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Aim 2: Flavonoid Scavenger</t>
+          <t>Aim 2: ROS Scavenger Specialist</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>O=c1cc(-c2ccc(O)c(O)c2)oc2cc(F)cc(O)c12</t>
+          <t>COc1ccc(-c2cc(=O)c3c(O)cc(O)cc3o2)cc1O</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>288.23</v>
+        <v>300.27</v>
       </c>
       <c r="E63" t="n">
-        <v>2.72</v>
+        <v>2.59</v>
       </c>
       <c r="F63" t="n">
-        <v>90.90000000000001</v>
+        <v>100.13</v>
       </c>
       <c r="G63" t="n">
         <v>3</v>
       </c>
       <c r="H63" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I63" t="n">
-        <v>-6.05</v>
+        <v>-6.7</v>
       </c>
       <c r="J63" t="n">
-        <v>3.123</v>
+        <v>2.997</v>
       </c>
       <c r="K63" t="n">
-        <v>18.89</v>
+        <v>20.08</v>
       </c>
       <c r="L63" t="inlineStr">
         <is>
@@ -3660,42 +3660,42 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CHEMBL247484</t>
+          <t>CHEMBL469752</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Aim 2: Flavonoid Scavenger</t>
+          <t>Aim 2: ROS Scavenger Specialist</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>O=c1cc(-c2cc(O)c(O)c(O)c2)oc2cc(O)cc(O)c12</t>
+          <t>COc1cc(O)c2c(=O)c(O)c(-c3ccc(O)c(O)c3)oc2c1</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>302.24</v>
+        <v>316.27</v>
       </c>
       <c r="E64" t="n">
-        <v>1.99</v>
+        <v>2.29</v>
       </c>
       <c r="F64" t="n">
-        <v>131.36</v>
+        <v>120.36</v>
       </c>
       <c r="G64" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H64" t="n">
         <v>7</v>
       </c>
       <c r="I64" t="n">
-        <v>-6.05</v>
+        <v>-6.7</v>
       </c>
       <c r="J64" t="n">
-        <v>4.963</v>
+        <v>3.794</v>
       </c>
       <c r="K64" t="n">
-        <v>30.03</v>
+        <v>25.42</v>
       </c>
       <c r="L64" t="inlineStr">
         <is>
@@ -3711,42 +3711,42 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CHEMBL151</t>
+          <t>CHEMBL243677</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Aim 2: Flavonoid Scavenger</t>
+          <t>Aim 2: ROS Scavenger Specialist</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>O=c1cc(-c2ccc(O)c(O)c2)oc2cc(O)cc(O)c12</t>
+          <t>O=c1cc(-c2ccc(O)c(O)c2)oc2cccc(O)c12</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>286.24</v>
+        <v>270.24</v>
       </c>
       <c r="E65" t="n">
-        <v>2.28</v>
+        <v>2.58</v>
       </c>
       <c r="F65" t="n">
-        <v>111.13</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="G65" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H65" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I65" t="n">
-        <v>-6.05</v>
+        <v>-6.7</v>
       </c>
       <c r="J65" t="n">
-        <v>4.192</v>
+        <v>3.33</v>
       </c>
       <c r="K65" t="n">
-        <v>25.36</v>
+        <v>22.31</v>
       </c>
       <c r="L65" t="inlineStr">
         <is>
@@ -3762,42 +3762,42 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CHEMBL3896909</t>
+          <t>CHEMBL43184</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Aim 2: Flavonoid Scavenger</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Oc1cc(O)c2c(=S)cc(-c3ccc(O)c(O)c3)oc2c1</t>
+          <t>Nc1c2ccccc2nc2ccccc12</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>302.31</v>
+        <v>194.24</v>
       </c>
       <c r="E66" t="n">
-        <v>3.65</v>
+        <v>2.97</v>
       </c>
       <c r="F66" t="n">
-        <v>94.06</v>
+        <v>38.91</v>
       </c>
       <c r="G66" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H66" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I66" t="n">
-        <v>-6.05</v>
+        <v>-6.7</v>
       </c>
       <c r="J66" t="n">
-        <v>3.969</v>
+        <v>0.772</v>
       </c>
       <c r="K66" t="n">
-        <v>24.01</v>
+        <v>5.17</v>
       </c>
       <c r="L66" t="inlineStr">
         <is>
@@ -3813,42 +3813,42 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CHEMBL117</t>
+          <t>CHEMBL357429</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Aim 2: Flavonoid Scavenger</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>O=c1cc(-c2ccccc2)oc2cc(O)cc(O)c12</t>
+          <t>Cc1ccc2nc3ccccc3c(N)c2c1</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>254.24</v>
+        <v>208.26</v>
       </c>
       <c r="E67" t="n">
-        <v>2.87</v>
+        <v>3.28</v>
       </c>
       <c r="F67" t="n">
-        <v>70.67</v>
+        <v>38.91</v>
       </c>
       <c r="G67" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H67" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I67" t="n">
-        <v>-6.05</v>
+        <v>-6.7</v>
       </c>
       <c r="J67" t="n">
-        <v>2.36</v>
+        <v>0.72</v>
       </c>
       <c r="K67" t="n">
-        <v>14.28</v>
+        <v>4.82</v>
       </c>
       <c r="L67" t="inlineStr">
         <is>
@@ -3864,42 +3864,42 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CHEMBL486407</t>
+          <t>CHEMBL343190</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Aim 2: Flavonoid Scavenger</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>O=c1cc(-c2ccc(F)cc2)oc2cc(O)cc(O)c12</t>
+          <t>Cc1cccc2c(N)c3ccccc3nc12</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>272.23</v>
+        <v>208.26</v>
       </c>
       <c r="E68" t="n">
-        <v>3.01</v>
+        <v>3.28</v>
       </c>
       <c r="F68" t="n">
-        <v>70.67</v>
+        <v>38.91</v>
       </c>
       <c r="G68" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H68" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I68" t="n">
-        <v>-6.05</v>
+        <v>-6.7</v>
       </c>
       <c r="J68" t="n">
-        <v>2.204</v>
+        <v>0.72</v>
       </c>
       <c r="K68" t="n">
-        <v>13.33</v>
+        <v>4.82</v>
       </c>
       <c r="L68" t="inlineStr">
         <is>
@@ -3915,42 +3915,42 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CHEMBL264037</t>
+          <t>CHEMBL146512</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Aim 2: Flavonoid Scavenger</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>O=c1cc(-c2ccc(Cl)cc2)oc2cc(O)cc(O)c12</t>
+          <t>Nc1c2ccccc2nc2cc(Cl)ccc12</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>288.69</v>
+        <v>228.68</v>
       </c>
       <c r="E69" t="n">
-        <v>3.52</v>
+        <v>3.62</v>
       </c>
       <c r="F69" t="n">
-        <v>70.67</v>
+        <v>38.91</v>
       </c>
       <c r="G69" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H69" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I69" t="n">
-        <v>-6.05</v>
+        <v>-6.7</v>
       </c>
       <c r="J69" t="n">
-        <v>2.078</v>
+        <v>0.656</v>
       </c>
       <c r="K69" t="n">
-        <v>12.57</v>
+        <v>4.4</v>
       </c>
       <c r="L69" t="inlineStr">
         <is>
@@ -3966,42 +3966,42 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CHEMBL167154</t>
+          <t>CHEMBL176543</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Aim 2: Flavonoid Scavenger</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Nc1ccc(-c2cc(=O)c3c(O)cc(O)cc3o2)cc1</t>
+          <t>CCN(CC)CCNc1c2ccccc2nc2ccccc12</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>269.26</v>
+        <v>293.41</v>
       </c>
       <c r="E70" t="n">
-        <v>2.45</v>
+        <v>4.14</v>
       </c>
       <c r="F70" t="n">
-        <v>96.69</v>
+        <v>28.16</v>
       </c>
       <c r="G70" t="n">
+        <v>1</v>
+      </c>
+      <c r="H70" t="n">
         <v>3</v>
       </c>
-      <c r="H70" t="n">
-        <v>5</v>
-      </c>
       <c r="I70" t="n">
-        <v>-6.05</v>
+        <v>-6.7</v>
       </c>
       <c r="J70" t="n">
-        <v>2.785</v>
+        <v>0.341</v>
       </c>
       <c r="K70" t="n">
-        <v>16.85</v>
+        <v>2.28</v>
       </c>
       <c r="L70" t="inlineStr">
         <is>
@@ -4017,42 +4017,42 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CHEMBL1821732</t>
+          <t>CHEMBL147657</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Aim 2: Flavonoid Scavenger</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>O=c1cc(-c2ccc(F)c(F)c2)oc2cc(O)cc(O)c12</t>
+          <t>Nc1c2ccccc2nc2ccc(Cl)cc12</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>290.22</v>
+        <v>228.68</v>
       </c>
       <c r="E71" t="n">
-        <v>3.15</v>
+        <v>3.62</v>
       </c>
       <c r="F71" t="n">
-        <v>70.67</v>
+        <v>38.91</v>
       </c>
       <c r="G71" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H71" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I71" t="n">
-        <v>-6.05</v>
+        <v>-6.7</v>
       </c>
       <c r="J71" t="n">
-        <v>2.067</v>
+        <v>0.656</v>
       </c>
       <c r="K71" t="n">
-        <v>12.51</v>
+        <v>4.4</v>
       </c>
       <c r="L71" t="inlineStr">
         <is>
@@ -4068,42 +4068,42 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CHEMBL457821</t>
+          <t>CHEMBL1596095</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Aim 2: Flavonoid Scavenger</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>O=c1cc(-c2cccc(O)c2)oc2cc(O)cc(O)c12</t>
+          <t>Fc1ccc(-c2nc3ccccc3[nH]2)cc1</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>270.24</v>
+        <v>212.23</v>
       </c>
       <c r="E72" t="n">
-        <v>2.58</v>
+        <v>3.37</v>
       </c>
       <c r="F72" t="n">
-        <v>90.90000000000001</v>
+        <v>28.68</v>
       </c>
       <c r="G72" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H72" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I72" t="n">
-        <v>-6.05</v>
+        <v>-6.7</v>
       </c>
       <c r="J72" t="n">
-        <v>3.33</v>
+        <v>0.471</v>
       </c>
       <c r="K72" t="n">
-        <v>20.15</v>
+        <v>3.16</v>
       </c>
       <c r="L72" t="inlineStr">
         <is>
@@ -4119,42 +4119,42 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CHEMBL1822222</t>
+          <t>CHEMBL2283280</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Aim 2: Flavonoid Scavenger</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>O=c1cc(-c2ccc(I)cc2)oc2cc(O)cc(O)c12</t>
+          <t>Cc1ccc(-c2nc3ccccc3[nH]2)cc1</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>380.14</v>
+        <v>208.26</v>
       </c>
       <c r="E73" t="n">
-        <v>3.48</v>
+        <v>3.54</v>
       </c>
       <c r="F73" t="n">
-        <v>70.67</v>
+        <v>28.68</v>
       </c>
       <c r="G73" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H73" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I73" t="n">
-        <v>-6.05</v>
+        <v>-6.7</v>
       </c>
       <c r="J73" t="n">
-        <v>1.578</v>
+        <v>0.48</v>
       </c>
       <c r="K73" t="n">
-        <v>9.550000000000001</v>
+        <v>3.22</v>
       </c>
       <c r="L73" t="inlineStr">
         <is>
@@ -4170,42 +4170,42 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CHEMBL471181</t>
+          <t>CHEMBL1883643</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Aim 2: Flavonoid Scavenger</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>O=c1cc(-c2ccc(Br)cc2)oc2cc(O)cc(O)c12</t>
+          <t>Cc1c2ccccc2nc2ccccc12</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>333.14</v>
+        <v>193.25</v>
       </c>
       <c r="E74" t="n">
-        <v>3.63</v>
+        <v>3.7</v>
       </c>
       <c r="F74" t="n">
-        <v>70.67</v>
+        <v>12.89</v>
       </c>
       <c r="G74" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H74" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I74" t="n">
-        <v>-6.05</v>
+        <v>-6.7</v>
       </c>
       <c r="J74" t="n">
-        <v>1.801</v>
+        <v>0.517</v>
       </c>
       <c r="K74" t="n">
-        <v>10.9</v>
+        <v>3.46</v>
       </c>
       <c r="L74" t="inlineStr">
         <is>
@@ -4221,42 +4221,42 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CHEMBL511458</t>
+          <t>CHEMBL153535</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Aim 2: Flavonoid Scavenger</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Oc1cc(O)c2c(c1)oc(-c1cc(O)c(O)c(O)c1)c(O)c2=O</t>
+          <t>c1ccc(-c2nc3ccccc3[nH]2)cc1</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>318.24</v>
+        <v>194.24</v>
       </c>
       <c r="E75" t="n">
-        <v>1.69</v>
+        <v>3.23</v>
       </c>
       <c r="F75" t="n">
-        <v>151.59</v>
+        <v>28.68</v>
       </c>
       <c r="G75" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H75" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="I75" t="n">
-        <v>-6.05</v>
+        <v>-6.7</v>
       </c>
       <c r="J75" t="n">
-        <v>5.656</v>
+        <v>0.515</v>
       </c>
       <c r="K75" t="n">
-        <v>34.22</v>
+        <v>3.45</v>
       </c>
       <c r="L75" t="inlineStr">
         <is>
@@ -4272,42 +4272,42 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CHEMBL243677</t>
+          <t>CHEMBL531708</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Aim 2: Flavonoid Scavenger</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>O=c1cc(-c2ccc(O)c(O)c2)oc2cccc(O)c12</t>
+          <t>Cl.Nc1c2ccccc2nc2cc([N+](=O)[O-])ccc12</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>270.24</v>
+        <v>275.69</v>
       </c>
       <c r="E76" t="n">
-        <v>2.58</v>
+        <v>3.3</v>
       </c>
       <c r="F76" t="n">
-        <v>90.90000000000001</v>
+        <v>82.05</v>
       </c>
       <c r="G76" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H76" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I76" t="n">
-        <v>-6.05</v>
+        <v>-6.7</v>
       </c>
       <c r="J76" t="n">
-        <v>3.33</v>
+        <v>0.544</v>
       </c>
       <c r="K76" t="n">
-        <v>20.15</v>
+        <v>3.64</v>
       </c>
       <c r="L76" t="inlineStr">
         <is>
@@ -4323,42 +4323,42 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CHEMBL5398631</t>
+          <t>CHEMBL581508</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Aim 2: Flavonoid Scavenger</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>O=C(O)c1cc(-c2cc(=O)c3c(O)cc(O)cc3o2)ccc1O</t>
+          <t>Nc1c2ccccc2nc2cc(C(F)(F)F)ccc12</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>314.25</v>
+        <v>262.23</v>
       </c>
       <c r="E77" t="n">
-        <v>2.27</v>
+        <v>3.99</v>
       </c>
       <c r="F77" t="n">
-        <v>128.2</v>
+        <v>38.91</v>
       </c>
       <c r="G77" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H77" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I77" t="n">
-        <v>-6</v>
+        <v>-6.7</v>
       </c>
       <c r="J77" t="n">
-        <v>2.864</v>
+        <v>0.572</v>
       </c>
       <c r="K77" t="n">
-        <v>17.18</v>
+        <v>3.83</v>
       </c>
       <c r="L77" t="inlineStr">
         <is>
@@ -4374,42 +4374,42 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CHEMBL183745</t>
+          <t>CHEMBL1308088</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Aim 2: Flavonoid Scavenger</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>COc1cc(O)c2c(=O)cc(-c3ccc(O)c(O)c3)oc2c1</t>
+          <t>Cl.Nc1c2ccccc2nc2ccccc12.O</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>300.27</v>
+        <v>248.71</v>
       </c>
       <c r="E78" t="n">
-        <v>2.59</v>
+        <v>2.57</v>
       </c>
       <c r="F78" t="n">
-        <v>100.13</v>
+        <v>70.41</v>
       </c>
       <c r="G78" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H78" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I78" t="n">
-        <v>-6</v>
+        <v>-6.7</v>
       </c>
       <c r="J78" t="n">
-        <v>2.997</v>
+        <v>0.603</v>
       </c>
       <c r="K78" t="n">
-        <v>17.98</v>
+        <v>4.04</v>
       </c>
       <c r="L78" t="inlineStr">
         <is>
@@ -4425,42 +4425,42 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CHEMBL214321</t>
+          <t>CHEMBL1534413</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Aim 2: Flavonoid Scavenger</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>COc1cc(-c2cc(=O)c3c(O)cc(O)cc3o2)ccc1O</t>
+          <t>Clc1ccc2[nH]c(-c3ccccc3)nc2c1</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>300.27</v>
+        <v>228.68</v>
       </c>
       <c r="E79" t="n">
-        <v>2.59</v>
+        <v>3.88</v>
       </c>
       <c r="F79" t="n">
-        <v>100.13</v>
+        <v>28.68</v>
       </c>
       <c r="G79" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H79" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I79" t="n">
-        <v>-6</v>
+        <v>-6.7</v>
       </c>
       <c r="J79" t="n">
-        <v>2.997</v>
+        <v>0.437</v>
       </c>
       <c r="K79" t="n">
-        <v>17.98</v>
+        <v>2.93</v>
       </c>
       <c r="L79" t="inlineStr">
         <is>
@@ -4476,42 +4476,42 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CHEMBL90568</t>
+          <t>CHEMBL2180144</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Aim 2: Flavonoid Scavenger</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>COc1ccc(-c2cc(=O)c3c(O)cc(O)cc3o2)cc1O</t>
+          <t>Clc1c2ccccc2nc2ccccc12</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>300.27</v>
+        <v>213.67</v>
       </c>
       <c r="E80" t="n">
-        <v>2.59</v>
+        <v>4.04</v>
       </c>
       <c r="F80" t="n">
-        <v>100.13</v>
+        <v>12.89</v>
       </c>
       <c r="G80" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H80" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I80" t="n">
-        <v>-6</v>
+        <v>-6.7</v>
       </c>
       <c r="J80" t="n">
-        <v>2.997</v>
+        <v>0.468</v>
       </c>
       <c r="K80" t="n">
-        <v>17.98</v>
+        <v>3.14</v>
       </c>
       <c r="L80" t="inlineStr">
         <is>
@@ -4527,42 +4527,42 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CHEMBL1277701</t>
+          <t>CHEMBL268354</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Aim 2: Flavonoid Scavenger</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>COc1cc(O)cc2oc(-c3ccc(O)c(O)c3)cc(=O)c12</t>
+          <t>Nc1nc(N)c2ccccc2n1</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>300.27</v>
+        <v>160.18</v>
       </c>
       <c r="E81" t="n">
-        <v>2.59</v>
+        <v>0.79</v>
       </c>
       <c r="F81" t="n">
-        <v>100.13</v>
+        <v>77.81999999999999</v>
       </c>
       <c r="G81" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H81" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I81" t="n">
-        <v>-6</v>
+        <v>-6.3</v>
       </c>
       <c r="J81" t="n">
-        <v>2.997</v>
+        <v>1.873</v>
       </c>
       <c r="K81" t="n">
-        <v>17.98</v>
+        <v>11.8</v>
       </c>
       <c r="L81" t="inlineStr">
         <is>
@@ -4571,34 +4571,34 @@
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>CHECK</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CHEMBL469752</t>
+          <t>CHEMBL459583</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Aim 2: Flavonoid Scavenger</t>
+          <t>Aim 2: ROS Scavenger Specialist</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>COc1cc(O)c2c(=O)c(O)c(-c3ccc(O)c(O)c3)oc2c1</t>
+          <t>COc1cc(/C=C/C(=O)c2cc(O)c(O)c(O)c2)cc(OC)c1O</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>316.27</v>
+        <v>332.31</v>
       </c>
       <c r="E82" t="n">
-        <v>2.29</v>
+        <v>2.42</v>
       </c>
       <c r="F82" t="n">
-        <v>120.36</v>
+        <v>116.45</v>
       </c>
       <c r="G82" t="n">
         <v>4</v>
@@ -4607,13 +4607,13 @@
         <v>7</v>
       </c>
       <c r="I82" t="n">
-        <v>-6</v>
+        <v>-6.3</v>
       </c>
       <c r="J82" t="n">
-        <v>3.794</v>
+        <v>3.611</v>
       </c>
       <c r="K82" t="n">
-        <v>22.76</v>
+        <v>22.75</v>
       </c>
       <c r="L82" t="inlineStr">
         <is>
@@ -4629,42 +4629,42 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CHEMBL117625</t>
+          <t>CHEMBL2006835</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Aim 2: Nitroxide/TEMPOL</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>CC1(C)CC(O)CC(C)(C)N1</t>
+          <t>Cl.NCCSSCc1ccccc1CSSCCN</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>157.26</v>
+        <v>357.04</v>
       </c>
       <c r="E83" t="n">
-        <v>1.29</v>
+        <v>3.79</v>
       </c>
       <c r="F83" t="n">
-        <v>32.26</v>
+        <v>52.04</v>
       </c>
       <c r="G83" t="n">
         <v>2</v>
       </c>
       <c r="H83" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="I83" t="n">
-        <v>-5.7</v>
+        <v>-5.9</v>
       </c>
       <c r="J83" t="n">
-        <v>0.636</v>
+        <v>0.28</v>
       </c>
       <c r="K83" t="n">
-        <v>3.63</v>
+        <v>1.65</v>
       </c>
       <c r="L83" t="inlineStr">
         <is>
@@ -4680,42 +4680,42 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CHEMBL459583</t>
+          <t>CHEMBL117625</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Aim 2: Polyphenol Scavenger</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>COc1cc(/C=C/C(=O)c2cc(O)c(O)c(O)c2)cc(OC)c1O</t>
+          <t>CC1(C)CC(O)CC(C)(C)N1</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>332.31</v>
+        <v>157.26</v>
       </c>
       <c r="E84" t="n">
-        <v>2.42</v>
+        <v>1.29</v>
       </c>
       <c r="F84" t="n">
-        <v>116.45</v>
+        <v>32.26</v>
       </c>
       <c r="G84" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H84" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I84" t="n">
-        <v>-5.65</v>
+        <v>-5.9</v>
       </c>
       <c r="J84" t="n">
-        <v>3.611</v>
+        <v>0.636</v>
       </c>
       <c r="K84" t="n">
-        <v>20.4</v>
+        <v>3.75</v>
       </c>
       <c r="L84" t="inlineStr">
         <is>
@@ -4736,7 +4736,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Aim 2: Aminothiol/Disulfide</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -4760,13 +4760,13 @@
         <v>3</v>
       </c>
       <c r="I85" t="n">
-        <v>-5.5</v>
+        <v>-5.9</v>
       </c>
       <c r="J85" t="n">
         <v>0.54</v>
       </c>
       <c r="K85" t="n">
-        <v>2.97</v>
+        <v>3.19</v>
       </c>
       <c r="L85" t="inlineStr">
         <is>
@@ -4782,24 +4782,24 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CHEMBL1256388</t>
+          <t>CHEMBL2009493</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Aim 2: Aminothiol/Disulfide</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Cl.NCCSSCCN</t>
+          <t>NCCSSCc1ccccc1CSSCCN</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>188.75</v>
+        <v>320.57</v>
       </c>
       <c r="E86" t="n">
-        <v>0.71</v>
+        <v>3.37</v>
       </c>
       <c r="F86" t="n">
         <v>52.04</v>
@@ -4808,16 +4808,16 @@
         <v>2</v>
       </c>
       <c r="H86" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I86" t="n">
-        <v>-5.25</v>
+        <v>-5.9</v>
       </c>
       <c r="J86" t="n">
-        <v>0.53</v>
+        <v>0.312</v>
       </c>
       <c r="K86" t="n">
-        <v>2.78</v>
+        <v>1.84</v>
       </c>
       <c r="L86" t="inlineStr">
         <is>
@@ -4826,7 +4826,7 @@
       </c>
       <c r="M86" t="inlineStr">
         <is>
-          <t>CHECK</t>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -4838,7 +4838,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Aim 2: Aminothiol/Disulfide</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -4862,13 +4862,13 @@
         <v>4</v>
       </c>
       <c r="I87" t="n">
-        <v>-5.25</v>
+        <v>-5.5</v>
       </c>
       <c r="J87" t="n">
         <v>0.657</v>
       </c>
       <c r="K87" t="n">
-        <v>3.45</v>
+        <v>3.61</v>
       </c>
       <c r="L87" t="inlineStr">
         <is>
@@ -4884,24 +4884,24 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>CHEMBL1594935</t>
+          <t>CHEMBL1256388</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Aim 2: Aminothiol/Disulfide</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Cl.Cl.NCCSSCCN</t>
+          <t>Cl.NCCSSCCN</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>225.21</v>
+        <v>188.75</v>
       </c>
       <c r="E88" t="n">
-        <v>1.13</v>
+        <v>0.71</v>
       </c>
       <c r="F88" t="n">
         <v>52.04</v>
@@ -4913,13 +4913,13 @@
         <v>4</v>
       </c>
       <c r="I88" t="n">
-        <v>-5.25</v>
+        <v>-5.5</v>
       </c>
       <c r="J88" t="n">
-        <v>0.444</v>
+        <v>0.53</v>
       </c>
       <c r="K88" t="n">
-        <v>2.33</v>
+        <v>2.92</v>
       </c>
       <c r="L88" t="inlineStr">
         <is>
@@ -4928,31 +4928,31 @@
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>CHECK</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CHEMBL2009493</t>
+          <t>CHEMBL1594935</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Aim 2: Aminothiol/Disulfide</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>NCCSSCc1ccccc1CSSCCN</t>
+          <t>Cl.Cl.NCCSSCCN</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>320.57</v>
+        <v>225.21</v>
       </c>
       <c r="E89" t="n">
-        <v>3.37</v>
+        <v>1.13</v>
       </c>
       <c r="F89" t="n">
         <v>52.04</v>
@@ -4961,16 +4961,16 @@
         <v>2</v>
       </c>
       <c r="H89" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I89" t="n">
-        <v>-5.2</v>
+        <v>-5.5</v>
       </c>
       <c r="J89" t="n">
-        <v>0.312</v>
+        <v>0.444</v>
       </c>
       <c r="K89" t="n">
-        <v>1.62</v>
+        <v>2.44</v>
       </c>
       <c r="L89" t="inlineStr">
         <is>
@@ -4986,24 +4986,24 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CHEMBL2006835</t>
+          <t>CHEMBL1979625</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Aim 2: Aminothiol/Disulfide</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Cl.NCCSSCc1ccccc1CSSCCN</t>
+          <t>Cl.NCCSSC/C=C\CSSCCN</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>357.04</v>
+        <v>306.98</v>
       </c>
       <c r="E90" t="n">
-        <v>3.79</v>
+        <v>2.64</v>
       </c>
       <c r="F90" t="n">
         <v>52.04</v>
@@ -5015,13 +5015,13 @@
         <v>6</v>
       </c>
       <c r="I90" t="n">
-        <v>-5.2</v>
+        <v>-5.5</v>
       </c>
       <c r="J90" t="n">
-        <v>0.28</v>
+        <v>0.326</v>
       </c>
       <c r="K90" t="n">
-        <v>1.46</v>
+        <v>1.79</v>
       </c>
       <c r="L90" t="inlineStr">
         <is>
@@ -5042,7 +5042,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Aim 2: Aminothiol/Disulfide</t>
+          <t>Moderate / Basal Profile</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -5066,13 +5066,13 @@
         <v>6</v>
       </c>
       <c r="I91" t="n">
-        <v>-5</v>
+        <v>-5.5</v>
       </c>
       <c r="J91" t="n">
         <v>0.37</v>
       </c>
       <c r="K91" t="n">
-        <v>1.85</v>
+        <v>2.04</v>
       </c>
       <c r="L91" t="inlineStr">
         <is>
@@ -5080,261 +5080,6 @@
         </is>
       </c>
       <c r="M91" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>CHEMBL1979625</t>
-        </is>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>Aim 2: Aminothiol/Disulfide</t>
-        </is>
-      </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>Cl.NCCSSC/C=C\CSSCCN</t>
-        </is>
-      </c>
-      <c r="D92" t="n">
-        <v>306.98</v>
-      </c>
-      <c r="E92" t="n">
-        <v>2.64</v>
-      </c>
-      <c r="F92" t="n">
-        <v>52.04</v>
-      </c>
-      <c r="G92" t="n">
-        <v>2</v>
-      </c>
-      <c r="H92" t="n">
-        <v>6</v>
-      </c>
-      <c r="I92" t="n">
-        <v>-5</v>
-      </c>
-      <c r="J92" t="n">
-        <v>0.326</v>
-      </c>
-      <c r="K92" t="n">
-        <v>1.63</v>
-      </c>
-      <c r="L92" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="M92" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>CHEMBL3215831</t>
-        </is>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>Aim 2: Aminothiol/Disulfide</t>
-        </is>
-      </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>Cl.Cl.NCCSSCCNC(=O)CCC(=O)NCCSSCCNC(=O)CCC(=O)NCCSSCCN</t>
-        </is>
-      </c>
-      <c r="D93" t="n">
-        <v>693.9</v>
-      </c>
-      <c r="E93" t="n">
-        <v>1.92</v>
-      </c>
-      <c r="F93" t="n">
-        <v>168.44</v>
-      </c>
-      <c r="G93" t="n">
-        <v>6</v>
-      </c>
-      <c r="H93" t="n">
-        <v>12</v>
-      </c>
-      <c r="I93" t="n">
-        <v>-4.25</v>
-      </c>
-      <c r="J93" t="n">
-        <v>0.144</v>
-      </c>
-      <c r="K93" t="n">
-        <v>0.61</v>
-      </c>
-      <c r="L93" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="M93" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>CHEMBL1851695</t>
-        </is>
-      </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>Aim 2: Aminothiol/Disulfide</t>
-        </is>
-      </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>NCCSSCCNC(=O)CCC(=O)NCCSSCCNC(=O)CCC(=O)NCCSSCCN</t>
-        </is>
-      </c>
-      <c r="D94" t="n">
-        <v>620.98</v>
-      </c>
-      <c r="E94" t="n">
-        <v>1.07</v>
-      </c>
-      <c r="F94" t="n">
-        <v>168.44</v>
-      </c>
-      <c r="G94" t="n">
-        <v>6</v>
-      </c>
-      <c r="H94" t="n">
-        <v>12</v>
-      </c>
-      <c r="I94" t="n">
-        <v>-4.25</v>
-      </c>
-      <c r="J94" t="n">
-        <v>0.161</v>
-      </c>
-      <c r="K94" t="n">
-        <v>0.68</v>
-      </c>
-      <c r="L94" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="M94" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t>CHEMBL3216486</t>
-        </is>
-      </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>Aim 2: Aminothiol/Disulfide</t>
-        </is>
-      </c>
-      <c r="C95" t="inlineStr">
-        <is>
-          <t>Cl.Cl.NCCSSCCNC(=O)CCCC(=O)NCCSSCCNC(=O)CCCC(=O)NCCSSCCN</t>
-        </is>
-      </c>
-      <c r="D95" t="n">
-        <v>721.96</v>
-      </c>
-      <c r="E95" t="n">
-        <v>2.7</v>
-      </c>
-      <c r="F95" t="n">
-        <v>168.44</v>
-      </c>
-      <c r="G95" t="n">
-        <v>6</v>
-      </c>
-      <c r="H95" t="n">
-        <v>12</v>
-      </c>
-      <c r="I95" t="n">
-        <v>-4.15</v>
-      </c>
-      <c r="J95" t="n">
-        <v>0.139</v>
-      </c>
-      <c r="K95" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="L95" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="M95" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="inlineStr">
-        <is>
-          <t>CHEMBL1851860</t>
-        </is>
-      </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>Aim 2: Aminothiol/Disulfide</t>
-        </is>
-      </c>
-      <c r="C96" t="inlineStr">
-        <is>
-          <t>NCCSSCCNC(=O)CCCC(=O)NCCSSCCNC(=O)CCCC(=O)NCCSSCCN</t>
-        </is>
-      </c>
-      <c r="D96" t="n">
-        <v>649.03</v>
-      </c>
-      <c r="E96" t="n">
-        <v>1.85</v>
-      </c>
-      <c r="F96" t="n">
-        <v>168.44</v>
-      </c>
-      <c r="G96" t="n">
-        <v>6</v>
-      </c>
-      <c r="H96" t="n">
-        <v>12</v>
-      </c>
-      <c r="I96" t="n">
-        <v>-4.15</v>
-      </c>
-      <c r="J96" t="n">
-        <v>0.154</v>
-      </c>
-      <c r="K96" t="n">
-        <v>0.64</v>
-      </c>
-      <c r="L96" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="M96" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>

</xml_diff>